<commit_message>
E-book Excel complet (8 chapitres) : captures régénérées une par une, couverture fidèle, 7 modèles bonus
- 58 cas tableur + scripts des chapitres 4 à 6 relancés un par un : 72 captures comparées, aucune différence dans celles du livre
- couverture : 35 prompts testés, 7 modèles Excel (au lieu de promesses non tenues)
- bonus/ : stock, paie, facture TVA, tontine, Mobile Money, tableau de bord, ventes du mois

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T8L22svZaEaGYSwza4q3Yc
</commit_message>
<xml_diff>
--- a/produits/preuves/sortie/c3-noms/c3-noms.xlsx
+++ b/produits/preuves/sortie/c3-noms/c3-noms.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="43">
   <si>
     <t xml:space="preserve">Client</t>
   </si>
@@ -44,9 +44,15 @@
     <t xml:space="preserve">6 77 12 34 56</t>
   </si>
   <si>
+    <t xml:space="preserve">+237677123456</t>
+  </si>
+  <si>
     <t xml:space="preserve">BORIS tchoumi</t>
   </si>
   <si>
+    <t xml:space="preserve">+237699887766</t>
+  </si>
+  <si>
     <t xml:space="preserve">carine FOTSO</t>
   </si>
   <si>
@@ -56,21 +62,24 @@
     <t xml:space="preserve">Aminatou Njoya</t>
   </si>
   <si>
-    <t xml:space="preserve">+237677123456</t>
-  </si>
-  <si>
     <t xml:space="preserve">Esther  Nkou</t>
   </si>
   <si>
     <t xml:space="preserve">00237 655 44 33 22</t>
   </si>
   <si>
+    <t xml:space="preserve">+237655443322</t>
+  </si>
+  <si>
     <t xml:space="preserve">Joël  ATANGANA</t>
   </si>
   <si>
     <t xml:space="preserve">+33 6 12 34 56 78</t>
   </si>
   <si>
+    <t xml:space="preserve">À vérifier</t>
+  </si>
+  <si>
     <t xml:space="preserve">boris Tchoumi</t>
   </si>
   <si>
@@ -89,24 +98,36 @@
     <t xml:space="preserve">(237) 691-234-567</t>
   </si>
   <si>
+    <t xml:space="preserve">+237691234567</t>
+  </si>
+  <si>
     <t xml:space="preserve">marie-claire EWANE</t>
   </si>
   <si>
     <t xml:space="preserve">237 670 55 66 77</t>
   </si>
   <si>
+    <t xml:space="preserve">+237670556677</t>
+  </si>
+  <si>
     <t xml:space="preserve">Hervé  KAMGA</t>
   </si>
   <si>
     <t xml:space="preserve">+237 6 99 00 11 22</t>
   </si>
   <si>
+    <t xml:space="preserve">+237699001122</t>
+  </si>
+  <si>
     <t xml:space="preserve">sandrine abena</t>
   </si>
   <si>
     <t xml:space="preserve">694 12 12 12</t>
   </si>
   <si>
+    <t xml:space="preserve">+237694121212</t>
+  </si>
+  <si>
     <t xml:space="preserve">FATIMA bello</t>
   </si>
   <si>
@@ -120,6 +141,9 @@
   </si>
   <si>
     <t xml:space="preserve">651 20 30 40</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+237651203040</t>
   </si>
 </sst>
 </file>
@@ -368,10 +392,13 @@
         <f aca="false">PROPER(TRIM(LOWER(A2)))</f>
         <v>Aminatou Njoya</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B3" s="0" t="n">
         <v>699887766</v>
@@ -380,142 +407,178 @@
         <f aca="false">PROPER(TRIM(LOWER(A3)))</f>
         <v>Boris Tchoumi</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C4" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A4)))</f>
         <v>Carine Fotso</v>
       </c>
+      <c r="D4" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="C5" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A5)))</f>
         <v>Aminatou Njoya</v>
       </c>
+      <c r="D5" s="1" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B6" s="0" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C6" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A6)))</f>
         <v>Esther Nkou</v>
       </c>
+      <c r="D6" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B7" s="0" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A7)))</f>
         <v>Joël Atangana</v>
       </c>
+      <c r="D7" s="0" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B8" s="0" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C8" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A8)))</f>
         <v>Boris Tchoumi</v>
       </c>
+      <c r="D8" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C9" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A9)))</f>
         <v>Pauline Ngo Bassa</v>
       </c>
+      <c r="D9" s="0" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="0" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B10" s="0" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C10" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A10)))</f>
         <v>Armand Mbarga</v>
       </c>
+      <c r="D10" s="1" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="0" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="B11" s="0" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C11" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A11)))</f>
         <v>Marie-Claire Ewane</v>
       </c>
+      <c r="D11" s="1" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="0" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B12" s="0" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="C12" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A12)))</f>
         <v>Hervé Kamga</v>
       </c>
+      <c r="D12" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="0" t="s">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B13" s="0" t="s">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="C13" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A13)))</f>
         <v>Sandrine Abena</v>
       </c>
+      <c r="D13" s="1" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="0" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="B14" s="0" t="s">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="C14" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A14)))</f>
         <v>Fatima Bello</v>
       </c>
+      <c r="D14" s="0" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="0" t="s">
-        <v>32</v>
+        <v>39</v>
       </c>
       <c r="B15" s="0" t="n">
         <v>699112233</v>
@@ -524,17 +587,23 @@
         <f aca="false">PROPER(TRIM(LOWER(A15)))</f>
         <v>Carine Fotso</v>
       </c>
+      <c r="D15" s="1" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="0" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="B16" s="0" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C16" s="0" t="str">
         <f aca="false">PROPER(TRIM(LOWER(A16)))</f>
         <v>Paul Ebode</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>